<commit_message>
Refactor: Sync Excel data, implement refresh button and visual refinements
</commit_message>
<xml_diff>
--- a/public/indicadores_epq.xlsx
+++ b/public/indicadores_epq.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\00 - PROYECTOS\app_dashboard_epq\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\00 - PROYECTOS\app_dashboard_epq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F683761E-5FCF-4600-8179-ECA2D376EC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCFBB3BC-729A-44AC-8223-B3A4D9CC700A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{9696E92E-FDFD-499D-9B6F-124374ADE829}"/>
   </bookViews>
@@ -1271,7 +1271,7 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares 2" xfId="1" xr:uid="{A26D7901-07CC-410F-A5A6-C7E9FD29608C}"/>
-    <cellStyle name="Millares 2 2" xfId="2" xr:uid="{FBE42FAF-3BBB-4217-AD7D-0B0D7B676341}"/>
+    <cellStyle name="Millares 2 2" xfId="2" xr:uid="{3BEE46F0-0724-48CF-84FF-06FCADE08AF2}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>

</xml_diff>

<commit_message>
Finalización de dashboard EPQ: Reubicación de logo al header, corrección lógica de IANC y Continuidad de Aseo, mejoras de espaciado y adición de pie de página institucional.
</commit_message>
<xml_diff>
--- a/public/indicadores_epq.xlsx
+++ b/public/indicadores_epq.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\00 - PROYECTOS\app_dashboard_epq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\00 - PROYECTOS\app_dashboard_epq\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCFBB3BC-729A-44AC-8223-B3A4D9CC700A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A383430-09CF-4DCD-8E3E-A65DD982C83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{9696E92E-FDFD-499D-9B6F-124374ADE829}"/>
   </bookViews>
@@ -33,66 +33,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Sandra Mosquera</author>
-  </authors>
-  <commentList>
-    <comment ref="H74" authorId="0" shapeId="0" xr:uid="{5085F142-7249-49E5-A0A3-AC319C7A6B30}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Sandra Mosquera:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-No se encontró información</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I74" authorId="0" shapeId="0" xr:uid="{ABCB18D5-650D-4407-829B-818E80904D5C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Sandra Mosquera:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-No se encontró información</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="333">
   <si>
     <t>Fecha</t>
   </si>
@@ -878,42 +820,6 @@
   </si>
   <si>
     <t>72.84%</t>
-  </si>
-  <si>
-    <t>84.54%</t>
-  </si>
-  <si>
-    <t>68.64%</t>
-  </si>
-  <si>
-    <t>68.21%</t>
-  </si>
-  <si>
-    <t>73.87%</t>
-  </si>
-  <si>
-    <t>70.7%</t>
-  </si>
-  <si>
-    <t>77.37%</t>
-  </si>
-  <si>
-    <t>76.4%</t>
-  </si>
-  <si>
-    <t>69.29%</t>
-  </si>
-  <si>
-    <t>70.34%</t>
-  </si>
-  <si>
-    <t>73.29%</t>
-  </si>
-  <si>
-    <t>62.79%</t>
-  </si>
-  <si>
-    <t>72.03%</t>
   </si>
   <si>
     <t>71.43%</t>
@@ -1137,7 +1043,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1165,31 +1071,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1216,12 +1122,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1253,26 +1161,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="5">
     <cellStyle name="Millares 2" xfId="1" xr:uid="{A26D7901-07CC-410F-A5A6-C7E9FD29608C}"/>
     <cellStyle name="Millares 2 2" xfId="2" xr:uid="{3BEE46F0-0724-48CF-84FF-06FCADE08AF2}"/>
+    <cellStyle name="Millares 6" xfId="4" xr:uid="{FF0D1A71-5DFA-4317-9B11-566006A6B416}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1583,8 +1499,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D501CC65-3A1F-4EF3-B78F-11792D49ED3F}">
-  <dimension ref="A1:Q353"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D501CC65-3A1F-4EF3-B78F-11792D49ED3F}">
+  <dimension ref="A1:Q345"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="6" bestFit="1" customWidth="1"/>
@@ -1633,7 +1549,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -1665,7 +1581,7 @@
         <v>43861</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="C2" s="6">
         <v>18016</v>
@@ -1679,6 +1595,9 @@
       <c r="F2" s="5" t="s">
         <v>197</v>
       </c>
+      <c r="G2" s="5">
+        <v>0.72899999999999998</v>
+      </c>
       <c r="H2" s="6">
         <v>489332</v>
       </c>
@@ -1688,8 +1607,23 @@
       <c r="J2" s="6">
         <v>20</v>
       </c>
+      <c r="K2" s="17">
+        <v>0.16474402943193864</v>
+      </c>
+      <c r="L2" s="10">
+        <v>6789</v>
+      </c>
+      <c r="M2" s="17">
+        <v>0.96033070991334768</v>
+      </c>
+      <c r="N2" s="10">
+        <v>36240</v>
+      </c>
       <c r="O2" s="6">
         <v>2101</v>
+      </c>
+      <c r="P2" s="16">
+        <v>0.99309999999999998</v>
       </c>
       <c r="Q2" s="6">
         <v>2482</v>
@@ -1700,7 +1634,7 @@
         <v>43890</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="C3" s="6">
         <v>18247</v>
@@ -1714,6 +1648,9 @@
       <c r="F3" s="7">
         <v>0</v>
       </c>
+      <c r="G3" s="5">
+        <v>0.73099999999999998</v>
+      </c>
       <c r="H3" s="6">
         <v>465109</v>
       </c>
@@ -1723,8 +1660,23 @@
       <c r="J3" s="6">
         <v>18</v>
       </c>
+      <c r="K3" s="17">
+        <v>0.16374323567829818</v>
+      </c>
+      <c r="L3" s="10">
+        <v>6771</v>
+      </c>
+      <c r="M3" s="17">
+        <v>0.95970066372266438</v>
+      </c>
+      <c r="N3" s="10">
+        <v>36293</v>
+      </c>
       <c r="O3" s="6">
         <v>21418</v>
+      </c>
+      <c r="P3" s="16">
+        <v>1</v>
       </c>
       <c r="Q3" s="6">
         <v>2304</v>
@@ -1735,7 +1687,7 @@
         <v>43921</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="C4" s="6">
         <v>18751</v>
@@ -1749,6 +1701,9 @@
       <c r="F4" s="5" t="s">
         <v>198</v>
       </c>
+      <c r="G4" s="5">
+        <v>0.7288</v>
+      </c>
       <c r="H4" s="6">
         <v>548499</v>
       </c>
@@ -1758,8 +1713,23 @@
       <c r="J4" s="6">
         <v>15</v>
       </c>
+      <c r="K4" s="17">
+        <v>0.16274740956753739</v>
+      </c>
+      <c r="L4" s="10">
+        <v>6752</v>
+      </c>
+      <c r="M4" s="17">
+        <v>0.97838879066944617</v>
+      </c>
+      <c r="N4" s="10">
+        <v>37078</v>
+      </c>
       <c r="O4" s="6">
         <v>2053</v>
+      </c>
+      <c r="P4" s="16">
+        <v>1</v>
       </c>
       <c r="Q4" s="6">
         <v>2226</v>
@@ -1770,7 +1740,7 @@
         <v>43951</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="C5" s="6">
         <v>18914</v>
@@ -1784,6 +1754,9 @@
       <c r="F5" s="7">
         <v>0</v>
       </c>
+      <c r="G5" s="5">
+        <v>0.72619999999999996</v>
+      </c>
       <c r="H5" s="6">
         <v>565206</v>
       </c>
@@ -1793,8 +1766,23 @@
       <c r="J5" s="6">
         <v>14</v>
       </c>
+      <c r="K5" s="17">
+        <v>0.16256111901961998</v>
+      </c>
+      <c r="L5" s="10">
+        <v>6759</v>
+      </c>
+      <c r="M5" s="17">
+        <v>0.9782499934170682</v>
+      </c>
+      <c r="N5" s="10">
+        <v>37151</v>
+      </c>
       <c r="O5" s="6">
         <v>1992</v>
+      </c>
+      <c r="P5" s="16">
+        <v>1</v>
       </c>
       <c r="Q5" s="6">
         <v>1865</v>
@@ -1819,6 +1807,9 @@
       <c r="F6" s="7">
         <v>0</v>
       </c>
+      <c r="G6" s="5">
+        <v>0.72799999999999998</v>
+      </c>
       <c r="H6" s="6">
         <v>620748</v>
       </c>
@@ -1828,8 +1819,23 @@
       <c r="J6" s="6">
         <v>17</v>
       </c>
+      <c r="K6" s="17">
+        <v>0.16187683284457477</v>
+      </c>
+      <c r="L6" s="10">
+        <v>6751</v>
+      </c>
+      <c r="M6" s="17">
+        <v>0.97469651584423778</v>
+      </c>
+      <c r="N6" s="10">
+        <v>37095</v>
+      </c>
       <c r="O6" s="6">
         <v>2097</v>
+      </c>
+      <c r="P6" s="16">
+        <v>0.99450000000000005</v>
       </c>
       <c r="Q6" s="6">
         <v>2048</v>
@@ -1840,7 +1846,7 @@
         <v>44012</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="C7" s="6">
         <v>18992</v>
@@ -1854,6 +1860,9 @@
       <c r="F7" s="5" t="s">
         <v>199</v>
       </c>
+      <c r="G7" s="5">
+        <v>0.72970000000000002</v>
+      </c>
       <c r="H7" s="6">
         <v>601924</v>
       </c>
@@ -1863,8 +1872,23 @@
       <c r="J7" s="6">
         <v>17</v>
       </c>
+      <c r="K7" s="17">
+        <v>0.15959477768198055</v>
+      </c>
+      <c r="L7" s="10">
+        <v>6690</v>
+      </c>
+      <c r="M7" s="17">
+        <v>0.96557329767429667</v>
+      </c>
+      <c r="N7" s="10">
+        <v>36826</v>
+      </c>
       <c r="O7" s="6">
         <v>2036</v>
+      </c>
+      <c r="P7" s="16">
+        <v>1</v>
       </c>
       <c r="Q7" s="6">
         <v>2305</v>
@@ -1875,7 +1899,7 @@
         <v>44043</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="C8" s="6">
         <v>19028</v>
@@ -1889,6 +1913,9 @@
       <c r="F8" s="5" t="s">
         <v>200</v>
       </c>
+      <c r="G8" s="5">
+        <v>0.73309999999999997</v>
+      </c>
       <c r="H8" s="6">
         <v>630786</v>
       </c>
@@ -1898,8 +1925,23 @@
       <c r="J8" s="6">
         <v>17</v>
       </c>
+      <c r="K8" s="17">
+        <v>0.15895199189114476</v>
+      </c>
+      <c r="L8" s="10">
+        <v>6682</v>
+      </c>
+      <c r="M8" s="17">
+        <v>0.96386708529565668</v>
+      </c>
+      <c r="N8" s="10">
+        <v>36839</v>
+      </c>
       <c r="O8" s="6">
         <v>2169</v>
+      </c>
+      <c r="P8" s="16">
+        <v>1</v>
       </c>
       <c r="Q8" s="6">
         <v>2256</v>
@@ -1910,7 +1952,7 @@
         <v>44074</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="C9" s="6">
         <v>18844</v>
@@ -1924,6 +1966,9 @@
       <c r="F9" s="5" t="s">
         <v>201</v>
       </c>
+      <c r="G9" s="5">
+        <v>0.73040000000000005</v>
+      </c>
       <c r="H9" s="6">
         <v>518726</v>
       </c>
@@ -1933,8 +1978,23 @@
       <c r="J9" s="6">
         <v>14</v>
       </c>
+      <c r="K9" s="17">
+        <v>0.15527912249525094</v>
+      </c>
+      <c r="L9" s="10">
+        <v>6575</v>
+      </c>
+      <c r="M9" s="17">
+        <v>0.9551186653089998</v>
+      </c>
+      <c r="N9" s="10">
+        <v>36582</v>
+      </c>
       <c r="O9" s="6">
         <v>2096</v>
+      </c>
+      <c r="P9" s="16">
+        <v>1</v>
       </c>
       <c r="Q9" s="6">
         <v>2484</v>
@@ -1945,7 +2005,7 @@
         <v>44104</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="C10" s="6">
         <v>18892</v>
@@ -1959,6 +2019,9 @@
       <c r="F10" s="5" t="s">
         <v>202</v>
       </c>
+      <c r="G10" s="5">
+        <v>0.72899999999999998</v>
+      </c>
       <c r="H10" s="6">
         <v>485982</v>
       </c>
@@ -1968,8 +2031,23 @@
       <c r="J10" s="6">
         <v>13</v>
       </c>
+      <c r="K10" s="17">
+        <v>0.15486414621473762</v>
+      </c>
+      <c r="L10" s="10">
+        <v>6574</v>
+      </c>
+      <c r="M10" s="17">
+        <v>0.95294669376270125</v>
+      </c>
+      <c r="N10" s="10">
+        <v>36576</v>
+      </c>
       <c r="O10" s="6">
         <v>2179</v>
+      </c>
+      <c r="P10" s="16">
+        <v>1</v>
       </c>
       <c r="Q10" s="6">
         <v>2483</v>
@@ -1980,7 +2058,7 @@
         <v>44135</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="C11" s="6">
         <v>19224</v>
@@ -1994,6 +2072,9 @@
       <c r="F11" s="5" t="s">
         <v>203</v>
       </c>
+      <c r="G11" s="5">
+        <v>0.72809999999999997</v>
+      </c>
       <c r="H11" s="6">
         <v>502492</v>
       </c>
@@ -2003,8 +2084,23 @@
       <c r="J11" s="6">
         <v>14</v>
       </c>
+      <c r="K11" s="17">
+        <v>0.15414634146341463</v>
+      </c>
+      <c r="L11" s="10">
+        <v>6563</v>
+      </c>
+      <c r="M11" s="17">
+        <v>0.96562930608636877</v>
+      </c>
+      <c r="N11" s="10">
+        <v>37141</v>
+      </c>
       <c r="O11" s="6">
         <v>2212</v>
+      </c>
+      <c r="P11" s="16">
+        <v>1</v>
       </c>
       <c r="Q11" s="6">
         <v>2603</v>
@@ -2015,7 +2111,7 @@
         <v>44165</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="C12" s="6">
         <v>19216</v>
@@ -2029,6 +2125,9 @@
       <c r="F12" s="5" t="s">
         <v>204</v>
       </c>
+      <c r="G12" s="5">
+        <v>0.73229999999999995</v>
+      </c>
       <c r="H12" s="6">
         <v>482872</v>
       </c>
@@ -2038,8 +2137,23 @@
       <c r="J12" s="6">
         <v>14</v>
       </c>
+      <c r="K12" s="17">
+        <v>0.15373620023721907</v>
+      </c>
+      <c r="L12" s="10">
+        <v>6562</v>
+      </c>
+      <c r="M12" s="17">
+        <v>0.96339248650892484</v>
+      </c>
+      <c r="N12" s="10">
+        <v>37133</v>
+      </c>
       <c r="O12" s="6">
         <v>2151</v>
+      </c>
+      <c r="P12" s="16">
+        <v>1</v>
       </c>
       <c r="Q12" s="6">
         <v>2614</v>
@@ -2050,7 +2164,7 @@
         <v>44196</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="C13" s="6">
         <v>19281</v>
@@ -2064,6 +2178,9 @@
       <c r="F13" s="5" t="s">
         <v>205</v>
       </c>
+      <c r="G13" s="5">
+        <v>0.72230000000000005</v>
+      </c>
       <c r="H13" s="6">
         <v>549638</v>
       </c>
@@ -2073,8 +2190,23 @@
       <c r="J13" s="6">
         <v>14</v>
       </c>
+      <c r="K13" s="17">
+        <v>0.1533280747527456</v>
+      </c>
+      <c r="L13" s="10">
+        <v>6561</v>
+      </c>
+      <c r="M13" s="17">
+        <v>0.96212297734627805</v>
+      </c>
+      <c r="N13" s="10">
+        <v>37162</v>
+      </c>
       <c r="O13" s="6">
         <v>2189</v>
+      </c>
+      <c r="P13" s="16">
+        <v>1</v>
       </c>
       <c r="Q13" s="6">
         <v>2916</v>
@@ -2085,7 +2217,7 @@
         <v>44227</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="C14" s="6">
         <v>19287</v>
@@ -2098,6 +2230,9 @@
       </c>
       <c r="F14" s="5" t="s">
         <v>206</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0.76305629802847585</v>
       </c>
       <c r="H14" s="8">
         <v>525813</v>
@@ -2135,7 +2270,7 @@
         <v>44255</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="C15" s="6">
         <v>19336</v>
@@ -2148,6 +2283,9 @@
       </c>
       <c r="F15" s="7">
         <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0.76305629802847585</v>
       </c>
       <c r="H15" s="8">
         <v>468276</v>
@@ -2185,7 +2323,7 @@
         <v>44286</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="C16" s="6">
         <v>19406</v>
@@ -2198,6 +2336,9 @@
       </c>
       <c r="F16" s="5" t="s">
         <v>207</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0.76305629802847585</v>
       </c>
       <c r="H16" s="8">
         <v>532832</v>
@@ -2235,7 +2376,7 @@
         <v>44316</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="C17" s="6">
         <v>19399</v>
@@ -2248,6 +2389,9 @@
       </c>
       <c r="F17" s="5" t="s">
         <v>208</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0.76305629802847585</v>
       </c>
       <c r="H17" s="8">
         <v>489792</v>
@@ -2285,7 +2429,7 @@
         <v>44347</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="C18" s="6">
         <v>19509</v>
@@ -2298,6 +2442,9 @@
       </c>
       <c r="F18" s="7">
         <v>0</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0.76305629802847585</v>
       </c>
       <c r="H18" s="8">
         <v>538920</v>
@@ -2335,7 +2482,7 @@
         <v>44377</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="C19" s="6">
         <v>19613</v>
@@ -2348,6 +2495,9 @@
       </c>
       <c r="F19" s="5" t="s">
         <v>209</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0.76591052148231975</v>
       </c>
       <c r="H19" s="8">
         <v>535718</v>
@@ -2385,7 +2535,7 @@
         <v>44408</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="C20" s="6">
         <v>19597</v>
@@ -2398,6 +2548,9 @@
       </c>
       <c r="F20" s="7">
         <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0.76116653945359403</v>
       </c>
       <c r="H20" s="8">
         <v>504470</v>
@@ -2435,7 +2588,7 @@
         <v>44439</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="C21" s="6">
         <v>19729</v>
@@ -2448,6 +2601,9 @@
       </c>
       <c r="F21" s="5" t="s">
         <v>210</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0.76468898996493828</v>
       </c>
       <c r="H21" s="8">
         <v>510323</v>
@@ -2485,7 +2641,7 @@
         <v>44469</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="C22" s="6">
         <v>19739</v>
@@ -2498,6 +2654,9 @@
       </c>
       <c r="F22" s="7">
         <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0.76736333014381297</v>
       </c>
       <c r="H22" s="8">
         <v>494455</v>
@@ -2535,7 +2694,7 @@
         <v>44500</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="C23" s="6">
         <v>19741</v>
@@ -2548,6 +2707,9 @@
       </c>
       <c r="F23" s="7">
         <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0.76933591479994834</v>
       </c>
       <c r="H23" s="8">
         <v>497618</v>
@@ -2585,7 +2747,7 @@
         <v>44530</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="C24" s="6">
         <v>19721</v>
@@ -2598,6 +2760,9 @@
       </c>
       <c r="F24" s="5" t="s">
         <v>211</v>
+      </c>
+      <c r="G24" s="5">
+        <v>0.76853471663547879</v>
       </c>
       <c r="H24" s="8">
         <v>481273</v>
@@ -2635,7 +2800,7 @@
         <v>44561</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="C25" s="6">
         <v>19735</v>
@@ -2648,6 +2813,9 @@
       </c>
       <c r="F25" s="7">
         <v>0</v>
+      </c>
+      <c r="G25" s="5">
+        <v>0.7712753863288071</v>
       </c>
       <c r="H25" s="8">
         <v>478847</v>
@@ -2685,7 +2853,7 @@
         <v>44592</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="C26" s="6">
         <v>19733</v>
@@ -2738,7 +2906,7 @@
         <v>44620</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="C27" s="6">
         <v>19769</v>
@@ -2791,7 +2959,7 @@
         <v>44651</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="C28" s="6">
         <v>19887</v>
@@ -2844,7 +3012,7 @@
         <v>44681</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="C29" s="6">
         <v>19890</v>
@@ -2897,7 +3065,7 @@
         <v>44712</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="C30" s="6">
         <v>19887</v>
@@ -2950,7 +3118,7 @@
         <v>44742</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="C31" s="6">
         <v>19893</v>
@@ -3003,7 +3171,7 @@
         <v>44773</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C32" s="6">
         <v>19897</v>
@@ -3056,7 +3224,7 @@
         <v>44804</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="C33" s="6">
         <v>19898</v>
@@ -3109,7 +3277,7 @@
         <v>44834</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="C34" s="6">
         <v>19888</v>
@@ -3162,7 +3330,7 @@
         <v>44865</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="C35" s="6">
         <v>19942</v>
@@ -3215,7 +3383,7 @@
         <v>44895</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C36" s="6">
         <v>19961</v>
@@ -3268,7 +3436,7 @@
         <v>44926</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C37" s="6">
         <v>20093</v>
@@ -3321,7 +3489,7 @@
         <v>44957</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="C38" s="6">
         <v>20127</v>
@@ -3374,7 +3542,7 @@
         <v>44985</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="C39" s="6">
         <v>20224</v>
@@ -3427,7 +3595,7 @@
         <v>45016</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="C40" s="6">
         <v>20301</v>
@@ -3480,7 +3648,7 @@
         <v>45046</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="C41" s="6">
         <v>20884</v>
@@ -3586,7 +3754,7 @@
         <v>45107</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="C43" s="6">
         <v>21185</v>
@@ -3639,7 +3807,7 @@
         <v>45138</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C44" s="6">
         <v>21210</v>
@@ -3692,7 +3860,7 @@
         <v>45169</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="C45" s="6">
         <v>21238</v>
@@ -3745,7 +3913,7 @@
         <v>45199</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C46" s="6">
         <v>21266</v>
@@ -3798,7 +3966,7 @@
         <v>45230</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="C47" s="6">
         <v>21287</v>
@@ -3851,7 +4019,7 @@
         <v>45260</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C48" s="6">
         <v>21293</v>
@@ -3904,7 +4072,7 @@
         <v>45291</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="C49" s="6">
         <v>21299</v>
@@ -3957,7 +4125,7 @@
         <v>45322</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="C50" s="6">
         <v>21153</v>
@@ -4010,7 +4178,7 @@
         <v>45351</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C51" s="6">
         <v>21181</v>
@@ -4063,7 +4231,7 @@
         <v>45382</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C52" s="6">
         <v>21216</v>
@@ -4116,7 +4284,7 @@
         <v>45412</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C53" s="6">
         <v>21233</v>
@@ -4169,7 +4337,7 @@
         <v>45443</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="C54" s="6">
         <v>21261</v>
@@ -4222,7 +4390,7 @@
         <v>45473</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="C55" s="6">
         <v>21280</v>
@@ -4275,7 +4443,7 @@
         <v>45504</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="C56" s="6">
         <v>21317</v>
@@ -4328,7 +4496,7 @@
         <v>45535</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="C57" s="6">
         <v>21379</v>
@@ -4381,7 +4549,7 @@
         <v>45565</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="C58" s="6">
         <v>21506</v>
@@ -4434,7 +4602,7 @@
         <v>45596</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C59" s="6">
         <v>21532</v>
@@ -4487,7 +4655,7 @@
         <v>45626</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C60" s="6">
         <v>21569</v>
@@ -4540,7 +4708,7 @@
         <v>45657</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C61" s="6">
         <v>21690</v>
@@ -4588,639 +4756,639 @@
         <v>2834</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A62" s="4">
+    <row r="62" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="11">
         <v>45688</v>
       </c>
-      <c r="B62" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="C62" s="6">
+      <c r="B62" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="C62" s="13">
         <v>21811</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="E62" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F62" s="7">
+      <c r="F62" s="14">
         <v>0</v>
       </c>
-      <c r="G62" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="H62" s="8">
+      <c r="G62" s="12">
+        <v>0.74070000000000003</v>
+      </c>
+      <c r="H62" s="15">
         <v>674770</v>
       </c>
-      <c r="I62" s="8">
+      <c r="I62" s="15">
         <v>104350</v>
       </c>
-      <c r="J62" s="6" t="s">
+      <c r="J62" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="K62" s="5" t="s">
+      <c r="K62" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="L62" s="6">
+      <c r="L62" s="13">
         <v>6560</v>
       </c>
-      <c r="M62" s="5" t="s">
+      <c r="M62" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="N62" s="6">
+      <c r="N62" s="13">
         <v>42207</v>
       </c>
-      <c r="O62" s="6">
+      <c r="O62" s="13">
         <v>2725</v>
       </c>
-      <c r="P62" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q62" s="6">
+      <c r="P62" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q62" s="13">
         <v>2597</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A63" s="4">
+    <row r="63" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="11">
         <v>45716</v>
       </c>
-      <c r="B63" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="C63" s="6">
+      <c r="B63" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="C63" s="13">
         <v>21891</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D63" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="E63" s="5" t="s">
+      <c r="E63" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F63" s="7">
+      <c r="F63" s="14">
         <v>0</v>
       </c>
-      <c r="G63" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="H63" s="8">
+      <c r="G63" s="12">
+        <v>0.74239999999999995</v>
+      </c>
+      <c r="H63" s="15">
         <v>603868</v>
       </c>
-      <c r="I63" s="8">
+      <c r="I63" s="15">
         <v>189349</v>
       </c>
-      <c r="J63" s="6" t="s">
+      <c r="J63" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="K63" s="5" t="s">
+      <c r="K63" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="L63" s="6">
+      <c r="L63" s="13">
         <v>6559</v>
       </c>
-      <c r="M63" s="5" t="s">
+      <c r="M63" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="N63" s="6">
+      <c r="N63" s="13">
         <v>42367</v>
       </c>
-      <c r="O63" s="6">
+      <c r="O63" s="13">
         <v>2429</v>
       </c>
-      <c r="P63" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q63" s="6">
+      <c r="P63" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q63" s="13">
         <v>2306</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A64" s="4">
+    <row r="64" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="11">
         <v>45747</v>
       </c>
-      <c r="B64" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C64" s="6">
+      <c r="B64" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="C64" s="13">
         <v>21922</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="D64" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="E64" s="5" t="s">
+      <c r="E64" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F64" s="7">
+      <c r="F64" s="14">
         <v>0</v>
       </c>
-      <c r="G64" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="H64" s="8">
+      <c r="G64" s="12">
+        <v>0.73839999999999995</v>
+      </c>
+      <c r="H64" s="15">
         <v>644895</v>
       </c>
-      <c r="I64" s="8">
+      <c r="I64" s="15">
         <v>205011</v>
       </c>
-      <c r="J64" s="6" t="s">
+      <c r="J64" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="K64" s="5" t="s">
+      <c r="K64" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="L64" s="6">
+      <c r="L64" s="13">
         <v>6577</v>
       </c>
-      <c r="M64" s="5" t="s">
+      <c r="M64" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="N64" s="6">
+      <c r="N64" s="13">
         <v>42379</v>
       </c>
-      <c r="O64" s="6">
+      <c r="O64" s="13">
         <v>2645</v>
       </c>
-      <c r="P64" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q64" s="6">
+      <c r="P64" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q64" s="13">
         <v>2453</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A65" s="4">
+    <row r="65" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="11">
         <v>45777</v>
       </c>
-      <c r="B65" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C65" s="6">
+      <c r="B65" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="C65" s="13">
         <v>21989</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="D65" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="E65" s="5" t="s">
+      <c r="E65" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F65" s="7">
+      <c r="F65" s="14">
         <v>0</v>
       </c>
-      <c r="G65" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="H65" s="8">
+      <c r="G65" s="12">
+        <v>0.73809999999999998</v>
+      </c>
+      <c r="H65" s="15">
         <v>624382</v>
       </c>
-      <c r="I65" s="8">
+      <c r="I65" s="15">
         <v>163162</v>
       </c>
-      <c r="J65" s="6" t="s">
+      <c r="J65" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="K65" s="5" t="s">
+      <c r="K65" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="L65" s="6">
+      <c r="L65" s="13">
         <v>6577</v>
       </c>
-      <c r="M65" s="5" t="s">
+      <c r="M65" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="N65" s="6">
+      <c r="N65" s="13">
         <v>42499</v>
       </c>
-      <c r="O65" s="6">
+      <c r="O65" s="13">
         <v>2624</v>
       </c>
-      <c r="P65" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q65" s="6">
+      <c r="P65" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q65" s="13">
         <v>2425</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A66" s="4">
+    <row r="66" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="11">
         <v>45808</v>
       </c>
-      <c r="B66" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C66" s="6">
+      <c r="B66" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="C66" s="13">
         <v>22059</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="E66" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F66" s="7">
+      <c r="F66" s="14">
         <v>0</v>
       </c>
-      <c r="G66" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="H66" s="8">
+      <c r="G66" s="12">
+        <v>0.73709999999999998</v>
+      </c>
+      <c r="H66" s="15">
         <v>653034</v>
       </c>
-      <c r="I66" s="8">
+      <c r="I66" s="15">
         <v>191357</v>
       </c>
-      <c r="J66" s="6" t="s">
+      <c r="J66" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="K66" s="5" t="s">
+      <c r="K66" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="L66" s="6">
+      <c r="L66" s="13">
         <v>6578</v>
       </c>
-      <c r="M66" s="5" t="s">
+      <c r="M66" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="N66" s="6">
+      <c r="N66" s="13">
         <v>42642</v>
       </c>
-      <c r="O66" s="6">
+      <c r="O66" s="13">
         <v>2725</v>
       </c>
-      <c r="P66" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q66" s="6">
+      <c r="P66" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q66" s="13">
         <v>2608</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A67" s="4">
+    <row r="67" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="11">
         <v>45838</v>
       </c>
-      <c r="B67" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="C67" s="6">
+      <c r="B67" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="C67" s="13">
         <v>22056</v>
       </c>
-      <c r="D67" s="5" t="s">
+      <c r="D67" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="E67" s="5" t="s">
+      <c r="E67" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F67" s="7">
+      <c r="F67" s="14">
         <v>0</v>
       </c>
-      <c r="G67" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="H67" s="8">
+      <c r="G67" s="12">
+        <v>0.7399</v>
+      </c>
+      <c r="H67" s="15">
         <v>653983</v>
       </c>
-      <c r="I67" s="8">
+      <c r="I67" s="15">
         <v>147980</v>
       </c>
-      <c r="J67" s="6" t="s">
+      <c r="J67" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="K67" s="5" t="s">
+      <c r="K67" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="L67" s="6">
+      <c r="L67" s="13">
         <v>6555</v>
       </c>
-      <c r="M67" s="5" t="s">
+      <c r="M67" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="N67" s="6">
+      <c r="N67" s="13">
         <v>42805</v>
       </c>
-      <c r="O67" s="6">
+      <c r="O67" s="13">
         <v>2546</v>
       </c>
-      <c r="P67" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q67" s="6">
+      <c r="P67" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q67" s="13">
         <v>2428</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A68" s="4">
+    <row r="68" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="11">
         <v>45869</v>
       </c>
-      <c r="B68" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="C68" s="6">
+      <c r="B68" s="12" t="s">
+        <v>320</v>
+      </c>
+      <c r="C68" s="13">
         <v>22126</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="D68" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="E68" s="5" t="s">
+      <c r="E68" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F68" s="7">
+      <c r="F68" s="14">
         <v>0</v>
       </c>
-      <c r="G68" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="H68" s="8">
+      <c r="G68" s="12">
+        <v>0.74229999999999996</v>
+      </c>
+      <c r="H68" s="15">
         <v>656212</v>
       </c>
-      <c r="I68" s="8">
+      <c r="I68" s="15">
         <v>154856</v>
       </c>
-      <c r="J68" s="6" t="s">
+      <c r="J68" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="K68" s="5" t="s">
+      <c r="K68" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="L68" s="6">
+      <c r="L68" s="13">
         <v>6550</v>
       </c>
-      <c r="M68" s="5" t="s">
+      <c r="M68" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="N68" s="6">
+      <c r="N68" s="13">
         <v>42934</v>
       </c>
-      <c r="O68" s="6">
+      <c r="O68" s="13">
         <v>2725</v>
       </c>
-      <c r="P68" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q68" s="6">
+      <c r="P68" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q68" s="13">
         <v>2755</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A69" s="4">
+    <row r="69" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="11">
         <v>45900</v>
       </c>
-      <c r="B69" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="C69" s="6">
+      <c r="B69" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="C69" s="13">
         <v>22120</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="D69" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="E69" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F69" s="7">
+      <c r="F69" s="14">
         <v>0</v>
       </c>
-      <c r="G69" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="H69" s="8">
+      <c r="G69" s="12">
+        <v>0.74039999999999995</v>
+      </c>
+      <c r="H69" s="15">
         <v>652023</v>
       </c>
-      <c r="I69" s="8">
+      <c r="I69" s="15">
         <v>200213</v>
       </c>
-      <c r="J69" s="6" t="s">
+      <c r="J69" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="K69" s="5" t="s">
+      <c r="K69" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L69" s="6">
+      <c r="L69" s="13">
         <v>6551</v>
       </c>
-      <c r="M69" s="5" t="s">
+      <c r="M69" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="N69" s="6">
+      <c r="N69" s="13">
         <v>42924</v>
       </c>
-      <c r="O69" s="6">
+      <c r="O69" s="13">
         <v>2725</v>
       </c>
-      <c r="P69" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q69" s="6">
+      <c r="P69" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q69" s="13">
         <v>2487</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A70" s="4">
+    <row r="70" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="11">
         <v>45930</v>
       </c>
-      <c r="B70" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C70" s="6">
+      <c r="B70" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="C70" s="13">
         <v>22128</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="E70" s="5" t="s">
+      <c r="E70" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F70" s="7">
+      <c r="F70" s="14">
         <v>0</v>
       </c>
-      <c r="G70" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="H70" s="8">
+      <c r="G70" s="12">
+        <v>0.73919999999999997</v>
+      </c>
+      <c r="H70" s="15">
         <v>642328</v>
       </c>
-      <c r="I70" s="8">
+      <c r="I70" s="15">
         <v>190495</v>
       </c>
-      <c r="J70" s="6" t="s">
+      <c r="J70" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K70" s="5" t="s">
+      <c r="K70" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="L70" s="6">
+      <c r="L70" s="13">
         <v>6551</v>
       </c>
-      <c r="M70" s="5" t="s">
+      <c r="M70" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="N70" s="6">
+      <c r="N70" s="13">
         <v>42939</v>
       </c>
-      <c r="O70" s="6">
+      <c r="O70" s="13">
         <v>2696</v>
       </c>
-      <c r="P70" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q70" s="6">
+      <c r="P70" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q70" s="13">
         <v>2585</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A71" s="4">
+    <row r="71" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="11">
         <v>45961</v>
       </c>
-      <c r="B71" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C71" s="6">
+      <c r="B71" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="C71" s="13">
         <v>22113</v>
       </c>
-      <c r="D71" s="5" t="s">
+      <c r="D71" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="E71" s="5" t="s">
+      <c r="E71" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F71" s="7">
+      <c r="F71" s="14">
         <v>0</v>
       </c>
-      <c r="G71" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="H71" s="8">
+      <c r="G71" s="12">
+        <v>0.73819999999999997</v>
+      </c>
+      <c r="H71" s="15">
         <v>696946</v>
       </c>
-      <c r="I71" s="8">
+      <c r="I71" s="15">
         <v>186133</v>
       </c>
-      <c r="J71" s="6" t="s">
+      <c r="J71" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="K71" s="5" t="s">
+      <c r="K71" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="L71" s="6">
+      <c r="L71" s="13">
         <v>6547</v>
       </c>
-      <c r="M71" s="5" t="s">
+      <c r="M71" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="N71" s="6">
+      <c r="N71" s="13">
         <v>42936</v>
       </c>
-      <c r="O71" s="6">
+      <c r="O71" s="13">
         <v>2725</v>
       </c>
-      <c r="P71" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q71" s="6">
+      <c r="P71" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q71" s="13">
         <v>2687</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A72" s="4">
+    <row r="72" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="11">
         <v>45991</v>
       </c>
-      <c r="B72" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="C72" s="6">
+      <c r="B72" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="C72" s="13">
         <v>22102</v>
       </c>
-      <c r="D72" s="5" t="s">
+      <c r="D72" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="E72" s="5" t="s">
+      <c r="E72" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="F72" s="7">
+      <c r="F72" s="14">
         <v>0</v>
       </c>
-      <c r="G72" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="H72" s="8">
+      <c r="G72" s="12">
+        <v>0.72770000000000001</v>
+      </c>
+      <c r="H72" s="15">
         <v>636589</v>
       </c>
-      <c r="I72" s="8">
+      <c r="I72" s="15">
         <v>236855</v>
       </c>
-      <c r="J72" s="6" t="s">
+      <c r="J72" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="K72" s="5" t="s">
+      <c r="K72" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="L72" s="6">
+      <c r="L72" s="13">
         <v>6546</v>
       </c>
-      <c r="M72" s="5" t="s">
+      <c r="M72" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="N72" s="6">
+      <c r="N72" s="13">
         <v>42938</v>
       </c>
-      <c r="O72" s="6">
+      <c r="O72" s="13">
         <v>2725</v>
       </c>
-      <c r="P72" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q72" s="6">
+      <c r="P72" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q72" s="13">
         <v>2618</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A73" s="4">
+    <row r="73" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="11">
         <v>46022</v>
       </c>
-      <c r="B73" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="C73" s="6">
+      <c r="B73" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="C73" s="13">
         <v>22100</v>
       </c>
-      <c r="D73" s="5" t="s">
+      <c r="D73" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="E73" s="5" t="s">
+      <c r="E73" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F73" s="7">
+      <c r="F73" s="14">
         <v>0</v>
       </c>
-      <c r="G73" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="H73" s="8">
+      <c r="G73" s="12">
+        <v>0.72370000000000001</v>
+      </c>
+      <c r="H73" s="15">
         <v>721002</v>
       </c>
-      <c r="I73" s="8">
+      <c r="I73" s="15">
         <v>201633</v>
       </c>
-      <c r="J73" s="6" t="s">
+      <c r="J73" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="K73" s="5" t="s">
+      <c r="K73" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="L73" s="6">
+      <c r="L73" s="13">
         <v>6547</v>
       </c>
-      <c r="M73" s="5" t="s">
+      <c r="M73" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="N73" s="6">
+      <c r="N73" s="13">
         <v>42954</v>
       </c>
-      <c r="O73" s="6">
+      <c r="O73" s="13">
         <v>2725</v>
       </c>
-      <c r="P73" s="7">
-        <v>1</v>
-      </c>
-      <c r="Q73" s="6">
+      <c r="P73" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q73" s="13">
         <v>3104</v>
       </c>
     </row>
@@ -5229,7 +5397,7 @@
         <v>46053</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C74" s="6">
         <v>22088</v>
@@ -5244,9 +5412,14 @@
         <v>0</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="H74" s="9"/>
+        <v>262</v>
+      </c>
+      <c r="H74" s="9">
+        <v>658437</v>
+      </c>
+      <c r="I74" s="6">
+        <v>173831</v>
+      </c>
       <c r="J74" s="6" t="s">
         <v>60</v>
       </c>
@@ -5277,7 +5450,7 @@
         <v>46081</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="C75" s="6">
         <v>22191</v>
@@ -5292,9 +5465,14 @@
         <v>0</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="H75" s="9"/>
+        <v>263</v>
+      </c>
+      <c r="H75" s="9">
+        <v>624657</v>
+      </c>
+      <c r="I75" s="6">
+        <v>207888</v>
+      </c>
       <c r="J75" s="6" t="s">
         <v>61</v>
       </c>
@@ -5321,55 +5499,55 @@
       </c>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A76" s="11">
+      <c r="A76" s="4">
         <v>46112</v>
       </c>
-      <c r="B76" s="12" t="s">
-        <v>340</v>
-      </c>
-      <c r="C76" s="13">
+      <c r="B76" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="C76" s="6">
         <v>22207</v>
       </c>
-      <c r="D76" s="12" t="s">
+      <c r="D76" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="E76" s="12" t="s">
+      <c r="E76" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F76" s="14">
+      <c r="F76" s="7">
         <v>0</v>
       </c>
-      <c r="G76" s="12" t="s">
-        <v>341</v>
-      </c>
-      <c r="H76" s="15">
+      <c r="G76" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="H76" s="8">
         <v>708274</v>
       </c>
-      <c r="I76" s="15">
+      <c r="I76" s="8">
         <v>205797</v>
       </c>
-      <c r="J76" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="K76" s="12" t="s">
-        <v>343</v>
-      </c>
-      <c r="L76" s="13">
+      <c r="J76" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="K76" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="L76" s="6">
         <v>6667</v>
       </c>
-      <c r="M76" s="12" t="s">
-        <v>344</v>
-      </c>
-      <c r="N76" s="13">
+      <c r="M76" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="N76" s="6">
         <v>44004</v>
       </c>
-      <c r="O76" s="13">
+      <c r="O76" s="6">
         <v>2725</v>
       </c>
-      <c r="P76" s="14">
-        <v>1</v>
-      </c>
-      <c r="Q76" s="13">
+      <c r="P76" s="7">
+        <v>1</v>
+      </c>
+      <c r="Q76" s="6">
         <v>2855</v>
       </c>
     </row>
@@ -5547,42 +5725,34 @@
     </row>
     <row r="111" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H111" s="9"/>
-      <c r="K111" s="7"/>
       <c r="P111" s="7"/>
     </row>
     <row r="112" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H112" s="9"/>
-      <c r="K112" s="7"/>
       <c r="P112" s="7"/>
     </row>
     <row r="113" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H113" s="9"/>
-      <c r="K113" s="7"/>
       <c r="P113" s="7"/>
     </row>
     <row r="114" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H114" s="9"/>
-      <c r="K114" s="7"/>
       <c r="P114" s="7"/>
     </row>
     <row r="115" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H115" s="9"/>
-      <c r="K115" s="7"/>
       <c r="P115" s="7"/>
     </row>
     <row r="116" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H116" s="9"/>
-      <c r="K116" s="7"/>
       <c r="P116" s="7"/>
     </row>
     <row r="117" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H117" s="9"/>
-      <c r="K117" s="7"/>
       <c r="P117" s="7"/>
     </row>
     <row r="118" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H118" s="9"/>
-      <c r="K118" s="7"/>
       <c r="P118" s="7"/>
     </row>
     <row r="119" spans="8:16" x14ac:dyDescent="0.3">
@@ -5727,35 +5897,35 @@
     </row>
     <row r="154" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H154" s="9"/>
-      <c r="P154" s="7"/>
+      <c r="P154" s="5"/>
     </row>
     <row r="155" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H155" s="9"/>
-      <c r="P155" s="7"/>
+      <c r="P155" s="5"/>
     </row>
     <row r="156" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H156" s="9"/>
-      <c r="P156" s="7"/>
+      <c r="P156" s="5"/>
     </row>
     <row r="157" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H157" s="9"/>
-      <c r="P157" s="7"/>
+      <c r="P157" s="5"/>
     </row>
     <row r="158" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H158" s="9"/>
-      <c r="P158" s="7"/>
+      <c r="P158" s="5"/>
     </row>
     <row r="159" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H159" s="9"/>
-      <c r="P159" s="7"/>
+      <c r="P159" s="5"/>
     </row>
     <row r="160" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H160" s="9"/>
-      <c r="P160" s="7"/>
+      <c r="P160" s="5"/>
     </row>
     <row r="161" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H161" s="9"/>
-      <c r="P161" s="7"/>
+      <c r="P161" s="5"/>
     </row>
     <row r="162" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H162" s="9"/>
@@ -5979,35 +6149,27 @@
     </row>
     <row r="217" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H217" s="9"/>
-      <c r="P217" s="5"/>
     </row>
     <row r="218" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H218" s="9"/>
-      <c r="P218" s="5"/>
     </row>
     <row r="219" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H219" s="9"/>
-      <c r="P219" s="5"/>
     </row>
     <row r="220" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H220" s="9"/>
-      <c r="P220" s="5"/>
     </row>
     <row r="221" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H221" s="9"/>
-      <c r="P221" s="5"/>
     </row>
     <row r="222" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H222" s="9"/>
-      <c r="P222" s="5"/>
     </row>
     <row r="223" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H223" s="9"/>
-      <c r="P223" s="5"/>
     </row>
     <row r="224" spans="8:16" x14ac:dyDescent="0.3">
       <c r="H224" s="9"/>
-      <c r="P224" s="5"/>
     </row>
     <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="9"/>
@@ -6371,34 +6533,9 @@
     </row>
     <row r="345" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H345" s="9"/>
-    </row>
-    <row r="346" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H346" s="9"/>
-    </row>
-    <row r="347" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H347" s="9"/>
-    </row>
-    <row r="348" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H348" s="9"/>
-    </row>
-    <row r="349" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H349" s="9"/>
-    </row>
-    <row r="350" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H350" s="9"/>
-    </row>
-    <row r="351" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H351" s="9"/>
-    </row>
-    <row r="352" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H352" s="9"/>
-    </row>
-    <row r="353" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H353" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ingreso de indicadores mes de Abril del 2026
</commit_message>
<xml_diff>
--- a/public/indicadores_epq.xlsx
+++ b/public/indicadores_epq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\00 - PROYECTOS\app_dashboard_epq\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A383430-09CF-4DCD-8E3E-A65DD982C83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C28BBD-E61A-4C4E-B36D-110F4E01440D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{9696E92E-FDFD-499D-9B6F-124374ADE829}"/>
   </bookViews>
@@ -5552,10 +5552,57 @@
       </c>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="H77" s="9"/>
-      <c r="K77" s="7"/>
-      <c r="M77" s="5"/>
-      <c r="P77" s="7"/>
+      <c r="A77" s="4">
+        <v>46142</v>
+      </c>
+      <c r="B77" s="5">
+        <v>0.50060000000000004</v>
+      </c>
+      <c r="C77" s="6">
+        <v>22204</v>
+      </c>
+      <c r="D77" s="5">
+        <v>0.93530000000000002</v>
+      </c>
+      <c r="E77" s="5">
+        <v>0.99819999999999998</v>
+      </c>
+      <c r="F77" s="7">
+        <v>0</v>
+      </c>
+      <c r="G77" s="5">
+        <v>0.71250000000000002</v>
+      </c>
+      <c r="H77" s="9">
+        <v>672152</v>
+      </c>
+      <c r="I77" s="6">
+        <v>196633</v>
+      </c>
+      <c r="J77" s="6">
+        <v>12.93</v>
+      </c>
+      <c r="K77" s="7">
+        <v>0.15029999999999999</v>
+      </c>
+      <c r="L77" s="6">
+        <v>6666</v>
+      </c>
+      <c r="M77" s="5">
+        <v>0.99209999999999998</v>
+      </c>
+      <c r="N77" s="6">
+        <v>44010</v>
+      </c>
+      <c r="O77" s="6">
+        <v>2725</v>
+      </c>
+      <c r="P77" s="7">
+        <v>1</v>
+      </c>
+      <c r="Q77" s="6">
+        <v>2715</v>
+      </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H78" s="9"/>

</xml_diff>